<commit_message>
Add Confluence source URLs to MQTT cells (release note + bus protocol spec)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0158eT26M2Dsi3JDmdySDo5Y
</commit_message>
<xml_diff>
--- a/en18031_asset_inventory/merged_v4_2026-10-02.xlsx
+++ b/en18031_asset_inventory/merged_v4_2026-10-02.xlsx
@@ -1000,7 +1000,8 @@
     <row r="49" ht="15.75" customHeight="1" s="42">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>1. MQTT reinstated. Retail-2026-04 release notes (Confluence CIED) and Jira ELD-2970 (Done, QA passed 6/23/26) show the MQTT client (AWS IoT, mqtt-glassos-bridge) shipping on embedded consoles. The 9/25/26 verbal retraction conflated the shipped Apple Watch MQTT integration with separate platform event-bus proposals. Rows 5, 11, 19, 25, 29, 34, 36, 42, Interfaces 11 and Where to Look 7 rewritten concisely against the shipped implementation.</t>
+          <t>1. MQTT reinstated. Retail-2026-04 release notes (Confluence CIED) and Jira ELD-2970 (Done, QA passed 6/23/26) show the MQTT client (AWS IoT, mqtt-glassos-bridge) shipping on embedded consoles. The 9/25/26 verbal retraction conflated the shipped Apple Watch MQTT integration with separate platform event-bus proposals. Rows 5, 11, 19, 25, 29, 34, 36, 42, Interfaces 11 and Where to Look 7 rewritten concisely against the shipped implementation.
+Sources: https://ifitdev.atlassian.net/wiki/spaces/CIED/pages/4918411394/2026-06-24+Retail-2026-04+Tier+3+Build#Apple-Watch-MQTT (release note, ELD-2970); https://ifitdev.atlassian.net/wiki/spaces/AV/pages/4734451720/Event+Bus+over+MQTT+v2 (bus protocol spec).</t>
         </is>
       </c>
     </row>
@@ -5500,7 +5501,8 @@
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>HTTPS/GraphQL confirmed (NIST 8259A: TLS only, cleartext disabled). MQTT confirmed shipped in Retail-2026-04 (ELD-2970, QA passed 6/23/26): AWS IoT Core, TLS on 443, per-session credentials from /v1/discover. Carries workout state and summaries including HR metrics (special category). OPEN: which bridge adapters are enabled in production, in particular WORKOUT_COMMANDS (phone-to-console start/pause/stop).</t>
+          <t>HTTPS/GraphQL confirmed (NIST 8259A: TLS only, cleartext disabled). MQTT confirmed shipped in Retail-2026-04 (ELD-2970, QA passed 6/23/26): AWS IoT Core, TLS on 443, per-session credentials from /v1/discover. Carries workout state and summaries including HR metrics (special category). OPEN: which bridge adapters are enabled in production, in particular WORKOUT_COMMANDS (phone-to-console start/pause/stop).
+Sources: https://ifitdev.atlassian.net/wiki/spaces/CIED/pages/4918411394/2026-06-24+Retail-2026-04+Tier+3+Build#Apple-Watch-MQTT (release note, ELD-2970); https://ifitdev.atlassian.net/wiki/spaces/AV/pages/4734451720/Event+Bus+over+MQTT+v2 (bus protocol spec).</t>
         </is>
       </c>
       <c r="N25" s="21" t="n"/>
@@ -6062,7 +6064,8 @@
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>CONFIRMED: heart rate crosses MQTT in both directions (production fixes ELD-3152/ELD-3153; Confluence 'Apple Watch — MQTT Transport'). Special-category health data (GDPR Art. 9), highest privacy priority on both platforms. Topics are user- and connection-scoped under a per-connection IAM policy. OPEN: confirm the AWS IoT custom authorizer validates the iFIT token on every connect.</t>
+          <t>CONFIRMED: heart rate crosses MQTT in both directions (production fixes ELD-3152/ELD-3153; Confluence 'Apple Watch — MQTT Transport'). Special-category health data (GDPR Art. 9), highest privacy priority on both platforms. Topics are user- and connection-scoped under a per-connection IAM policy. OPEN: confirm the AWS IoT custom authorizer validates the iFIT token on every connect.
+Sources: https://ifitdev.atlassian.net/wiki/spaces/CIED/pages/4918411394/2026-06-24+Retail-2026-04+Tier+3+Build#Apple-Watch-MQTT (release note, ELD-2970); https://ifitdev.atlassian.net/wiki/spaces/AV/pages/4734451720/Event+Bus+over+MQTT+v2 (bus protocol spec).</t>
         </is>
       </c>
       <c r="N34" s="21" t="n"/>
@@ -11980,7 +11983,8 @@
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Primary remote interface for nearly all Security, Network and Privacy assets. MQTT confirmed shipped in Retail-2026-04 (ELD-2970); see Confluence 'Apple Watch — MQTT Transport'. OPEN: production BridgeConfig adapter set.</t>
+          <t>Primary remote interface for nearly all Security, Network and Privacy assets. MQTT confirmed shipped in Retail-2026-04 (ELD-2970); see Confluence 'Apple Watch — MQTT Transport'. OPEN: production BridgeConfig adapter set.
+Sources: https://ifitdev.atlassian.net/wiki/spaces/CIED/pages/4918411394/2026-06-24+Retail-2026-04+Tier+3+Build#Apple-Watch-MQTT (release note, ELD-2970); https://ifitdev.atlassian.net/wiki/spaces/AV/pages/4734451720/Event+Bus+over+MQTT+v2 (bus protocol spec).</t>
         </is>
       </c>
     </row>
@@ -13252,7 +13256,8 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>iFIT: GraphQL HTTPS API (OkHttp) plus MQTT over TLS to AWS IoT (AWS CRT client, per-session credentials from /v1/discover). Certificate pinning status not confirmed; recommend explicit check.</t>
+          <t>iFIT: GraphQL HTTPS API (OkHttp) plus MQTT over TLS to AWS IoT (AWS CRT client, per-session credentials from /v1/discover). Certificate pinning status not confirmed; recommend explicit check.
+Sources: https://ifitdev.atlassian.net/wiki/spaces/CIED/pages/4918411394/2026-06-24+Retail-2026-04+Tier+3+Build#Apple-Watch-MQTT (release note, ELD-2970); https://ifitdev.atlassian.net/wiki/spaces/AV/pages/4734451720/Event+Bus+over+MQTT+v2 (bus protocol spec).</t>
         </is>
       </c>
     </row>

</xml_diff>